<commit_message>
Fix Excel snapshot: Cash CMA shows CHF rate (0.4%) instead of 3%
Task #290: The CMA Assumptions sheet in default-profile-snapshot.xlsx
showed Cash μ as the global BASE_SEED 3.0%, inconsistent with the rest
of the workbook which already uses RF_CHF (0.4%) for the cash sleeve
since the 2026-05 cash-mu-per-currency engine change.

Change:
- scripts/src/default-profile-snapshot.mts: inline cash.mu = 0.0040
  (with `/* RF.CHF */` comment) instead of 0.030. Inlined rather than
  referencing RF_CHF to avoid reordering the CMA/RF declarations.

Regenerated:
- scripts/output/default-profile-snapshot.xlsx
- artifacts/investment-lab/public/default-profile-snapshot.xlsx
  (the script writes both copies).

Sharpe for the Cash row recomputes automatically from the new μ.
No engine or other source files touched (per task out-of-scope).

Replit-Task-Id: 6b339a30-bb9b-4992-b62b-263acd828629
</commit_message>
<xml_diff>
--- a/artifacts/investment-lab/public/default-profile-snapshot.xlsx
+++ b/artifacts/investment-lab/public/default-profile-snapshot.xlsx
@@ -1703,14 +1703,14 @@
         <v>8</v>
       </c>
       <c r="C11" s="1">
-        <v>0.03</v>
+        <v>0.004</v>
       </c>
       <c r="D11" s="1">
         <v>0.005</v>
       </c>
       <c r="E11" s="10">
         <f>IF(D11&gt;0,(C11-F11)/D11,0)</f>
-        <v>5.199999999999999</v>
+        <v>0</v>
       </c>
       <c r="F11" s="1">
         <v>0.004</v>

</xml_diff>